<commit_message>
mark instances without labels and delete them
</commit_message>
<xml_diff>
--- a/data/requirements.xlsx
+++ b/data/requirements.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\scripts\hil\hil-test-case-gen\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08F510CF-6B31-4080-9739-E5FF06B99553}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{894AAE19-7E4B-46B1-9207-1EAF01924B8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
   <si>
     <t>requirement</t>
   </si>
@@ -92,9 +92,6 @@
     <t>The electronic control unit (ECU) must validate sensor input before executing throttle commands to prevent unintended acceleration</t>
   </si>
   <si>
-    <t>Upon detection of a sensor failure, the system must reduce engine power and notify the driver through a warning indicator</t>
-  </si>
-  <si>
     <t>The system must perform periodic performance checks on the accelerator pedal and throttle position sensors to ensure ongoing reliability</t>
   </si>
   <si>
@@ -137,9 +134,6 @@
     <t>The system must log data relevant to accelerator pedal operation to assist in troubleshooting and fault analysis</t>
   </si>
   <si>
-    <t>The system must adapt throttle adjustments based on environmental conditions detected by other vehicle sensors</t>
-  </si>
-  <si>
     <t>Vehicle acceleration must be linear and proportional to the displacement of the accelerator pedal to provide a smooth and controlled driving experience</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
     <t>Free play in the steering system must not exceed specified tolerances to prevent on-road steering imprecision</t>
   </si>
   <si>
-    <t>The steering system must react within a defined time frame from the driver's input to wheel turn</t>
-  </si>
-  <si>
     <t>Recirculating ball steering systems must provide consistent and predictable responses to steering inputs without undue lag or play</t>
   </si>
   <si>
@@ -167,9 +158,6 @@
     <t>Power steering systems, whether hydraulic or electronic, must operate effectively in a wide range of environmental conditions, including extreme temperatures</t>
   </si>
   <si>
-    <t>Steering systems must be capable of handling the expected range of loads without failure or excessive play developing over time</t>
-  </si>
-  <si>
     <t>In the absence of power assist, the manual steering effort required should comply with safety standards to ensure that the vehicle can still be controlled</t>
   </si>
   <si>
@@ -191,9 +179,6 @@
     <t>Data transmission from the steering angle sensor to various safety and assistance systems must be secured against unauthorized access and corruption</t>
   </si>
   <si>
-    <t>The vehicle dynamics control system must integrate steering stability data to actively manage the vehicle's handling characteristics, reducing the risk of oversteer and understeer</t>
-  </si>
-  <si>
     <t>The steering system should dynamically adjust to optimize cornering behavior, providing a balance between responsiveness and stability</t>
   </si>
   <si>
@@ -212,9 +197,6 @@
     <t>The system must detect any Steering Angle Sensor malfunction and report Diagnostic Trouble Codes (DTCs) to the vehicle’s diagnostic system promptly</t>
   </si>
   <si>
-    <t>The system must incorporate measures to automatically adjust for any detected sensor offset that could affect steering accuracy</t>
-  </si>
-  <si>
     <t>Upon detection of a fault condition, the system shall enter a fail-safe mode, maintaining limited operational capabilities to allow the vehicle to be steered to a safe stop</t>
   </si>
   <si>
@@ -266,9 +248,6 @@
     <t>The ABS shall monitor for irregular wheel speed variations that could indicate impending wheel lock-up or sensor faults</t>
   </si>
   <si>
-    <t>The ABS warning light must illuminate when a fault that affects braking performance is detected</t>
-  </si>
-  <si>
     <t>The vehicle control system shall counteract any vehicle handling issues due to wheel speed sensor faults, within system limits</t>
   </si>
   <si>
@@ -344,9 +323,6 @@
     <t>The electronic stability control (ESC) must detect and appropriately respond to oversteer conditions to maintain vehicle stability</t>
   </si>
   <si>
-    <t>Traction control systems must adapt to varying road surfaces to maintain tire grip and vehicle control</t>
-  </si>
-  <si>
     <t>Vehicle control systems must process yaw rate data in real-time to enable immediate corrective actions</t>
   </si>
   <si>
@@ -389,9 +365,6 @@
     <t>Vehicle suspension and steering systems must utilize yaw rate data to enhance road handling, especially in adverse conditions</t>
   </si>
   <si>
-    <t>The IMU must have redundancy to ensure that failure of one component does not lead to loss of vehicle stability control</t>
-  </si>
-  <si>
     <t>Vehicle telemetry systems must incorporate yaw rate sensor data to support advanced driver assistance systems (ADAS) and automated driving functions</t>
   </si>
   <si>
@@ -467,12 +440,6 @@
     <t>The power steering system should allow drivers to customize steering feedback settings according to personal preference, within safety limits</t>
   </si>
   <si>
-    <t>The hydraulic power steering system must maintain its integrity and not leak hydraulic fluid under nominal operating conditions</t>
-  </si>
-  <si>
-    <t>The system must monitor the temperature of the power steering fluid and take corrective action if temperatures exceed safe operating limits</t>
-  </si>
-  <si>
     <t>The electric power steering system must have a redundancy plan for critical components to maintain steering assistance in the event of partial system failure</t>
   </si>
   <si>
@@ -515,9 +482,6 @@
     <t>The power steering system must perform reliably over the vehicle's operational lifetime without degradation that impacts safety or control</t>
   </si>
   <si>
-    <t>EPS must function correctly within the full range of operational temperatures and conditions specified by the manufacturer</t>
-  </si>
-  <si>
     <t>The system must limit the steering effort required by the driver to a specified maximum under normal operating conditions</t>
   </si>
   <si>
@@ -548,9 +512,6 @@
     <t>Adaptive Cruise Control (ACC) must adjust the vehicle's speed based on both the steering angle and acceleration pedal position when a lane change is initiated</t>
   </si>
   <si>
-    <t>The vehicle control system shall automatically decelerate when a lane change in heavy traffic is detected without safe distances</t>
-  </si>
-  <si>
     <t>In case of wheel steering sensor failure, the system must revert to a fail-safe mode that allows for controlled and safe vehicle operation</t>
   </si>
   <si>
@@ -570,9 +531,6 @@
   </si>
   <si>
     <t>steering system assistance should be consistent across different steering angles and not impair the driver's ability to perform smooth cornering maneuvers</t>
-  </si>
-  <si>
-    <t>In the event of understeer, the system must adjust power distribution to aid in returning to the intended path</t>
   </si>
   <si>
     <t>The Power steering system must adjust the torque assist to ensure appropriate steering feedback and control</t>
@@ -788,8 +746,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9FFBFF32-7D69-4481-8A8B-5B21ABBD8279}" name="Table2" displayName="Table2" ref="A1:F210" totalsRowShown="0" dataDxfId="6">
-  <autoFilter ref="A1:F210" xr:uid="{9FFBFF32-7D69-4481-8A8B-5B21ABBD8279}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9FFBFF32-7D69-4481-8A8B-5B21ABBD8279}" name="Table2" displayName="Table2" ref="A1:F196" totalsRowShown="0" dataDxfId="6">
+  <autoFilter ref="A1:F196" xr:uid="{9FFBFF32-7D69-4481-8A8B-5B21ABBD8279}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{1CE00CE7-2033-4A6A-8A7F-6850FFBCD532}" name="requirement" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{C71C0448-D7DF-4CEE-BFD6-8E925377BEAE}" name="acceleration_pedal" dataDxfId="4"/>
@@ -1087,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F210"/>
+  <dimension ref="A1:F196"/>
   <sheetFormatPr defaultRowHeight="21" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="174.5546875" style="2" bestFit="1" customWidth="1"/>
@@ -1721,13 +1679,13 @@
     </row>
     <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
-        <v>36</v>
+        <v>159</v>
       </c>
       <c r="B32" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D32" s="1">
         <v>0</v>
@@ -1741,13 +1699,13 @@
     </row>
     <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
-        <v>37</v>
+        <v>160</v>
       </c>
       <c r="B33" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C33" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D33" s="1">
         <v>0</v>
@@ -1761,7 +1719,7 @@
     </row>
     <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
-        <v>172</v>
+        <v>36</v>
       </c>
       <c r="B34" s="1">
         <v>0</v>
@@ -1781,7 +1739,7 @@
     </row>
     <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
-        <v>173</v>
+        <v>37</v>
       </c>
       <c r="B35" s="1">
         <v>0</v>
@@ -1801,13 +1759,13 @@
     </row>
     <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
-        <v>38</v>
+        <v>161</v>
       </c>
       <c r="B36" s="1">
         <v>0</v>
       </c>
       <c r="C36" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D36" s="1">
         <v>0</v>
@@ -1816,18 +1774,18 @@
         <v>0</v>
       </c>
       <c r="F36" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
-        <v>39</v>
+        <v>162</v>
       </c>
       <c r="B37" s="1">
         <v>0</v>
       </c>
       <c r="C37" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D37" s="1">
         <v>0</v>
@@ -1836,18 +1794,18 @@
         <v>0</v>
       </c>
       <c r="F37" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
-        <v>40</v>
+        <v>163</v>
       </c>
       <c r="B38" s="1">
         <v>0</v>
       </c>
       <c r="C38" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D38" s="1">
         <v>0</v>
@@ -1856,12 +1814,12 @@
         <v>0</v>
       </c>
       <c r="F38" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
-        <v>174</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1">
         <v>0</v>
@@ -1881,13 +1839,13 @@
     </row>
     <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
-        <v>175</v>
+        <v>39</v>
       </c>
       <c r="B40" s="1">
         <v>0</v>
       </c>
       <c r="C40" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" s="1">
         <v>0</v>
@@ -1896,12 +1854,12 @@
         <v>0</v>
       </c>
       <c r="F40" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
-        <v>176</v>
+        <v>40</v>
       </c>
       <c r="B41" s="1">
         <v>0</v>
@@ -1921,13 +1879,13 @@
     </row>
     <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
-        <v>41</v>
+        <v>164</v>
       </c>
       <c r="B42" s="1">
         <v>0</v>
       </c>
       <c r="C42" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D42" s="1">
         <v>0</v>
@@ -1936,18 +1894,18 @@
         <v>0</v>
       </c>
       <c r="F42" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B43" s="1">
         <v>0</v>
       </c>
       <c r="C43" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D43" s="1">
         <v>0</v>
@@ -1956,18 +1914,18 @@
         <v>0</v>
       </c>
       <c r="F43" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B44" s="1">
         <v>0</v>
       </c>
       <c r="C44" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" s="1">
         <v>0</v>
@@ -1976,12 +1934,12 @@
         <v>0</v>
       </c>
       <c r="F44" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
-        <v>177</v>
+        <v>43</v>
       </c>
       <c r="B45" s="1">
         <v>0</v>
@@ -2027,7 +1985,7 @@
         <v>0</v>
       </c>
       <c r="C47" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D47" s="1">
         <v>0</v>
@@ -2036,7 +1994,7 @@
         <v>0</v>
       </c>
       <c r="F47" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -2061,7 +2019,7 @@
     </row>
     <row r="49" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
-        <v>47</v>
+        <v>165</v>
       </c>
       <c r="B49" s="1">
         <v>0</v>
@@ -2081,13 +2039,13 @@
     </row>
     <row r="50" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
-        <v>48</v>
+        <v>177</v>
       </c>
       <c r="B50" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C50" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D50" s="1">
         <v>0</v>
@@ -2101,7 +2059,7 @@
     </row>
     <row r="51" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B51" s="1">
         <v>0</v>
@@ -2121,7 +2079,7 @@
     </row>
     <row r="52" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B52" s="1">
         <v>0</v>
@@ -2141,7 +2099,7 @@
     </row>
     <row r="53" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
-        <v>178</v>
+        <v>49</v>
       </c>
       <c r="B53" s="1">
         <v>0</v>
@@ -2161,13 +2119,13 @@
     </row>
     <row r="54" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
-        <v>191</v>
+        <v>50</v>
       </c>
       <c r="B54" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C54" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D54" s="1">
         <v>0</v>
@@ -2367,10 +2325,10 @@
         <v>0</v>
       </c>
       <c r="C64" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D64" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E64" s="1">
         <v>0</v>
@@ -2387,10 +2345,10 @@
         <v>0</v>
       </c>
       <c r="C65" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D65" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E65" s="1">
         <v>0</v>
@@ -2407,10 +2365,10 @@
         <v>0</v>
       </c>
       <c r="C66" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D66" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E66" s="1">
         <v>0</v>
@@ -2427,10 +2385,10 @@
         <v>0</v>
       </c>
       <c r="C67" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D67" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E67" s="1">
         <v>0</v>
@@ -2447,10 +2405,10 @@
         <v>0</v>
       </c>
       <c r="C68" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D68" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E68" s="1">
         <v>0</v>
@@ -2467,10 +2425,10 @@
         <v>0</v>
       </c>
       <c r="C69" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D69" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E69" s="1">
         <v>0</v>
@@ -2764,13 +2722,13 @@
         <v>80</v>
       </c>
       <c r="B84" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C84" s="1">
         <v>0</v>
       </c>
       <c r="D84" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E84" s="1">
         <v>0</v>
@@ -2904,13 +2862,13 @@
         <v>87</v>
       </c>
       <c r="B91" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C91" s="1">
         <v>0</v>
       </c>
       <c r="D91" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E91" s="1">
         <v>0</v>
@@ -2930,10 +2888,10 @@
         <v>0</v>
       </c>
       <c r="D92" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E92" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F92" s="1">
         <v>0</v>
@@ -2950,10 +2908,10 @@
         <v>0</v>
       </c>
       <c r="D93" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E93" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F93" s="1">
         <v>0</v>
@@ -2970,10 +2928,10 @@
         <v>0</v>
       </c>
       <c r="D94" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E94" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F94" s="1">
         <v>0</v>
@@ -2990,10 +2948,10 @@
         <v>0</v>
       </c>
       <c r="D95" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E95" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F95" s="1">
         <v>0</v>
@@ -3010,10 +2968,10 @@
         <v>0</v>
       </c>
       <c r="D96" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E96" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F96" s="1">
         <v>0</v>
@@ -3030,10 +2988,10 @@
         <v>0</v>
       </c>
       <c r="D97" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E97" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F97" s="1">
         <v>0</v>
@@ -3050,10 +3008,10 @@
         <v>0</v>
       </c>
       <c r="D98" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E98" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F98" s="1">
         <v>0</v>
@@ -3221,7 +3179,7 @@
     </row>
     <row r="107" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
-        <v>179</v>
+        <v>103</v>
       </c>
       <c r="B107" s="1">
         <v>0</v>
@@ -3233,15 +3191,15 @@
         <v>0</v>
       </c>
       <c r="E107" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F107" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="108" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B108" s="1">
         <v>0</v>
@@ -3250,10 +3208,10 @@
         <v>0</v>
       </c>
       <c r="D108" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E108" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F108" s="1">
         <v>0</v>
@@ -3261,7 +3219,7 @@
     </row>
     <row r="109" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B109" s="1">
         <v>0</v>
@@ -3281,7 +3239,7 @@
     </row>
     <row r="110" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B110" s="1">
         <v>0</v>
@@ -3301,7 +3259,7 @@
     </row>
     <row r="111" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B111" s="1">
         <v>0</v>
@@ -3321,7 +3279,7 @@
     </row>
     <row r="112" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B112" s="1">
         <v>0</v>
@@ -3341,7 +3299,7 @@
     </row>
     <row r="113" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B113" s="1">
         <v>0</v>
@@ -3361,7 +3319,7 @@
     </row>
     <row r="114" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B114" s="1">
         <v>0</v>
@@ -3381,7 +3339,7 @@
     </row>
     <row r="115" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B115" s="1">
         <v>0</v>
@@ -3401,7 +3359,7 @@
     </row>
     <row r="116" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B116" s="1">
         <v>0</v>
@@ -3421,7 +3379,7 @@
     </row>
     <row r="117" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B117" s="1">
         <v>0</v>
@@ -3441,7 +3399,7 @@
     </row>
     <row r="118" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B118" s="1">
         <v>0</v>
@@ -3461,7 +3419,7 @@
     </row>
     <row r="119" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B119" s="1">
         <v>0</v>
@@ -3481,7 +3439,7 @@
     </row>
     <row r="120" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B120" s="1">
         <v>0</v>
@@ -3501,7 +3459,7 @@
     </row>
     <row r="121" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B121" s="1">
         <v>0</v>
@@ -3513,15 +3471,15 @@
         <v>0</v>
       </c>
       <c r="E121" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F121" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="122" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B122" s="1">
         <v>0</v>
@@ -3533,15 +3491,15 @@
         <v>0</v>
       </c>
       <c r="E122" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F122" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
-        <v>118</v>
+        <v>178</v>
       </c>
       <c r="B123" s="1">
         <v>0</v>
@@ -3553,10 +3511,10 @@
         <v>0</v>
       </c>
       <c r="E123" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F123" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="124" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -3573,10 +3531,10 @@
         <v>0</v>
       </c>
       <c r="E124" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F124" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="125" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -3593,10 +3551,10 @@
         <v>0</v>
       </c>
       <c r="E125" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F125" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="126" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -3613,10 +3571,10 @@
         <v>0</v>
       </c>
       <c r="E126" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F126" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -3633,10 +3591,10 @@
         <v>0</v>
       </c>
       <c r="E127" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F127" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="128" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
@@ -3653,15 +3611,15 @@
         <v>0</v>
       </c>
       <c r="E128" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F128" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A129" s="3" t="s">
-        <v>124</v>
+        <v>166</v>
       </c>
       <c r="B129" s="1">
         <v>0</v>
@@ -3673,15 +3631,15 @@
         <v>0</v>
       </c>
       <c r="E129" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F129" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="130" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
-        <v>125</v>
+        <v>167</v>
       </c>
       <c r="B130" s="1">
         <v>0</v>
@@ -3693,15 +3651,15 @@
         <v>0</v>
       </c>
       <c r="E130" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F130" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
-        <v>126</v>
+        <v>168</v>
       </c>
       <c r="B131" s="1">
         <v>0</v>
@@ -3721,7 +3679,7 @@
     </row>
     <row r="132" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B132" s="1">
         <v>0</v>
@@ -3741,7 +3699,7 @@
     </row>
     <row r="133" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
-        <v>192</v>
+        <v>125</v>
       </c>
       <c r="B133" s="1">
         <v>0</v>
@@ -3761,7 +3719,7 @@
     </row>
     <row r="134" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B134" s="1">
         <v>0</v>
@@ -3781,7 +3739,7 @@
     </row>
     <row r="135" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="B135" s="1">
         <v>0</v>
@@ -3801,7 +3759,7 @@
     </row>
     <row r="136" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="B136" s="1">
         <v>0</v>
@@ -3821,7 +3779,7 @@
     </row>
     <row r="137" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B137" s="1">
         <v>0</v>
@@ -3841,13 +3799,13 @@
     </row>
     <row r="138" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
-        <v>132</v>
+        <v>169</v>
       </c>
       <c r="B138" s="1">
         <v>0</v>
       </c>
       <c r="C138" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D138" s="1">
         <v>0</v>
@@ -3856,12 +3814,12 @@
         <v>0</v>
       </c>
       <c r="F138" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="139" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="B139" s="1">
         <v>0</v>
@@ -3881,7 +3839,7 @@
     </row>
     <row r="140" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
-        <v>181</v>
+        <v>130</v>
       </c>
       <c r="B140" s="1">
         <v>0</v>
@@ -3901,7 +3859,7 @@
     </row>
     <row r="141" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
-        <v>182</v>
+        <v>131</v>
       </c>
       <c r="B141" s="1">
         <v>0</v>
@@ -3921,7 +3879,7 @@
     </row>
     <row r="142" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A142" s="3" t="s">
-        <v>133</v>
+        <v>171</v>
       </c>
       <c r="B142" s="1">
         <v>0</v>
@@ -3941,13 +3899,13 @@
     </row>
     <row r="143" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A143" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B143" s="1">
         <v>0</v>
       </c>
       <c r="C143" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D143" s="1">
         <v>0</v>
@@ -3956,12 +3914,12 @@
         <v>0</v>
       </c>
       <c r="F143" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A144" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B144" s="1">
         <v>0</v>
@@ -3981,7 +3939,7 @@
     </row>
     <row r="145" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A145" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="B145" s="1">
         <v>0</v>
@@ -4001,7 +3959,7 @@
     </row>
     <row r="146" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A146" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="B146" s="1">
         <v>0</v>
@@ -4021,7 +3979,7 @@
     </row>
     <row r="147" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A147" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="B147" s="1">
         <v>0</v>
@@ -4041,13 +3999,13 @@
     </row>
     <row r="148" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A148" s="3" t="s">
-        <v>183</v>
+        <v>137</v>
       </c>
       <c r="B148" s="1">
         <v>0</v>
       </c>
       <c r="C148" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D148" s="1">
         <v>0</v>
@@ -4056,18 +4014,18 @@
         <v>0</v>
       </c>
       <c r="F148" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="149" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A149" s="3" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="B149" s="1">
         <v>0</v>
       </c>
       <c r="C149" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D149" s="1">
         <v>0</v>
@@ -4076,12 +4034,12 @@
         <v>0</v>
       </c>
       <c r="F149" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="150" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A150" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B150" s="1">
         <v>0</v>
@@ -4101,7 +4059,7 @@
     </row>
     <row r="151" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A151" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B151" s="1">
         <v>0</v>
@@ -4121,7 +4079,7 @@
     </row>
     <row r="152" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A152" s="3" t="s">
-        <v>185</v>
+        <v>140</v>
       </c>
       <c r="B152" s="1">
         <v>0</v>
@@ -4141,7 +4099,7 @@
     </row>
     <row r="153" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A153" s="3" t="s">
-        <v>141</v>
+        <v>173</v>
       </c>
       <c r="B153" s="1">
         <v>0</v>
@@ -4161,7 +4119,7 @@
     </row>
     <row r="154" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A154" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B154" s="1">
         <v>0</v>
@@ -4181,13 +4139,13 @@
     </row>
     <row r="155" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A155" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B155" s="1">
         <v>0</v>
       </c>
       <c r="C155" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D155" s="1">
         <v>0</v>
@@ -4196,12 +4154,12 @@
         <v>0</v>
       </c>
       <c r="F155" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A156" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B156" s="1">
         <v>0</v>
@@ -4221,7 +4179,7 @@
     </row>
     <row r="157" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A157" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B157" s="1">
         <v>0</v>
@@ -4241,7 +4199,7 @@
     </row>
     <row r="158" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A158" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B158" s="1">
         <v>0</v>
@@ -4261,7 +4219,7 @@
     </row>
     <row r="159" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A159" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B159" s="1">
         <v>0</v>
@@ -4281,7 +4239,7 @@
     </row>
     <row r="160" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A160" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B160" s="1">
         <v>0</v>
@@ -4301,13 +4259,13 @@
     </row>
     <row r="161" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A161" s="3" t="s">
-        <v>186</v>
+        <v>148</v>
       </c>
       <c r="B161" s="1">
         <v>0</v>
       </c>
       <c r="C161" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D161" s="1">
         <v>0</v>
@@ -4316,18 +4274,18 @@
         <v>0</v>
       </c>
       <c r="F161" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="162" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A162" s="3" t="s">
-        <v>149</v>
+        <v>174</v>
       </c>
       <c r="B162" s="1">
         <v>0</v>
       </c>
       <c r="C162" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D162" s="1">
         <v>0</v>
@@ -4336,12 +4294,12 @@
         <v>0</v>
       </c>
       <c r="F162" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="163" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A163" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B163" s="1">
         <v>0</v>
@@ -4361,7 +4319,7 @@
     </row>
     <row r="164" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A164" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B164" s="1">
         <v>0</v>
@@ -4381,13 +4339,13 @@
     </row>
     <row r="165" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A165" s="3" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
       <c r="B165" s="1">
         <v>0</v>
       </c>
       <c r="C165" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D165" s="1">
         <v>0</v>
@@ -4396,18 +4354,18 @@
         <v>0</v>
       </c>
       <c r="F165" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="166" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A166" s="3" t="s">
-        <v>152</v>
+        <v>175</v>
       </c>
       <c r="B166" s="1">
         <v>0</v>
       </c>
       <c r="C166" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D166" s="1">
         <v>0</v>
@@ -4416,18 +4374,18 @@
         <v>0</v>
       </c>
       <c r="F166" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="167" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A167" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B167" s="1">
         <v>0</v>
       </c>
       <c r="C167" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D167" s="1">
         <v>0</v>
@@ -4436,18 +4394,18 @@
         <v>0</v>
       </c>
       <c r="F167" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="168" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A168" s="3" t="s">
-        <v>154</v>
+        <v>181</v>
       </c>
       <c r="B168" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C168" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D168" s="1">
         <v>0</v>
@@ -4456,18 +4414,18 @@
         <v>0</v>
       </c>
       <c r="F168" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="169" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A169" s="3" t="s">
-        <v>155</v>
+        <v>182</v>
       </c>
       <c r="B169" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C169" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D169" s="1">
         <v>0</v>
@@ -4476,18 +4434,18 @@
         <v>0</v>
       </c>
       <c r="F169" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="170" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A170" s="3" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B170" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C170" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D170" s="1">
         <v>0</v>
@@ -4496,18 +4454,18 @@
         <v>0</v>
       </c>
       <c r="F170" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="171" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A171" s="3" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="B171" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C171" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D171" s="1">
         <v>0</v>
@@ -4516,18 +4474,18 @@
         <v>0</v>
       </c>
       <c r="F171" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="172" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A172" s="3" t="s">
-        <v>158</v>
+        <v>183</v>
       </c>
       <c r="B172" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C172" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D172" s="1">
         <v>0</v>
@@ -4536,18 +4494,18 @@
         <v>0</v>
       </c>
       <c r="F172" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="173" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A173" s="3" t="s">
-        <v>159</v>
+        <v>184</v>
       </c>
       <c r="B173" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C173" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D173" s="1">
         <v>0</v>
@@ -4556,15 +4514,15 @@
         <v>0</v>
       </c>
       <c r="F173" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A174" s="3" t="s">
-        <v>188</v>
+        <v>154</v>
       </c>
       <c r="B174" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C174" s="1">
         <v>1</v>
@@ -4581,7 +4539,7 @@
     </row>
     <row r="175" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A175" s="3" t="s">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="B175" s="1">
         <v>0</v>
@@ -4601,13 +4559,13 @@
     </row>
     <row r="176" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A176" s="3" t="s">
-        <v>161</v>
+        <v>185</v>
       </c>
       <c r="B176" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C176" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D176" s="1">
         <v>0</v>
@@ -4616,18 +4574,18 @@
         <v>0</v>
       </c>
       <c r="F176" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A177" s="3" t="s">
-        <v>162</v>
+        <v>186</v>
       </c>
       <c r="B177" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C177" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D177" s="1">
         <v>0</v>
@@ -4636,18 +4594,18 @@
         <v>0</v>
       </c>
       <c r="F177" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="178" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A178" s="3" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
       <c r="B178" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C178" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D178" s="1">
         <v>0</v>
@@ -4656,15 +4614,15 @@
         <v>0</v>
       </c>
       <c r="F178" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="179" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A179" s="3" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="B179" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C179" s="1">
         <v>1</v>
@@ -4681,13 +4639,13 @@
     </row>
     <row r="180" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A180" s="3" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="B180" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C180" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D180" s="1">
         <v>0</v>
@@ -4696,12 +4654,12 @@
         <v>0</v>
       </c>
       <c r="F180" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A181" s="3" t="s">
-        <v>195</v>
+        <v>156</v>
       </c>
       <c r="B181" s="1">
         <v>1</v>
@@ -4721,7 +4679,7 @@
     </row>
     <row r="182" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A182" s="3" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
       <c r="B182" s="1">
         <v>1</v>
@@ -4741,7 +4699,7 @@
     </row>
     <row r="183" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A183" s="3" t="s">
-        <v>164</v>
+        <v>200</v>
       </c>
       <c r="B183" s="1">
         <v>1</v>
@@ -4759,9 +4717,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A184" s="3" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="B184" s="1">
         <v>1</v>
@@ -4781,10 +4739,10 @@
     </row>
     <row r="185" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A185" s="3" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="B185" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C185" s="1">
         <v>1</v>
@@ -4801,7 +4759,7 @@
     </row>
     <row r="186" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A186" s="3" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
       <c r="B186" s="1">
         <v>1</v>
@@ -4821,7 +4779,7 @@
     </row>
     <row r="187" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A187" s="3" t="s">
-        <v>166</v>
+        <v>191</v>
       </c>
       <c r="B187" s="1">
         <v>1</v>
@@ -4841,13 +4799,13 @@
     </row>
     <row r="188" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A188" s="3" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B188" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C188" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D188" s="1">
         <v>0</v>
@@ -4856,12 +4814,12 @@
         <v>0</v>
       </c>
       <c r="F188" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A189" s="3" t="s">
-        <v>199</v>
+        <v>158</v>
       </c>
       <c r="B189" s="1">
         <v>1</v>
@@ -4881,7 +4839,7 @@
     </row>
     <row r="190" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A190" s="3" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B190" s="1">
         <v>1</v>
@@ -4901,7 +4859,7 @@
     </row>
     <row r="191" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A191" s="3" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B191" s="1">
         <v>1</v>
@@ -4921,7 +4879,7 @@
     </row>
     <row r="192" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A192" s="3" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="B192" s="1">
         <v>1</v>
@@ -4941,7 +4899,7 @@
     </row>
     <row r="193" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A193" s="3" t="s">
-        <v>167</v>
+        <v>196</v>
       </c>
       <c r="B193" s="1">
         <v>1</v>
@@ -4961,10 +4919,10 @@
     </row>
     <row r="194" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A194" s="3" t="s">
-        <v>168</v>
+        <v>197</v>
       </c>
       <c r="B194" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C194" s="1">
         <v>1</v>
@@ -4981,7 +4939,7 @@
     </row>
     <row r="195" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A195" s="3" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="B195" s="1">
         <v>1</v>
@@ -5001,7 +4959,7 @@
     </row>
     <row r="196" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A196" s="3" t="s">
-        <v>214</v>
+        <v>199</v>
       </c>
       <c r="B196" s="1">
         <v>1</v>
@@ -5016,286 +4974,6 @@
         <v>0</v>
       </c>
       <c r="F196" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="197" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A197" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="B197" s="1">
-        <v>1</v>
-      </c>
-      <c r="C197" s="1">
-        <v>1</v>
-      </c>
-      <c r="D197" s="1">
-        <v>0</v>
-      </c>
-      <c r="E197" s="1">
-        <v>0</v>
-      </c>
-      <c r="F197" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="198" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A198" s="3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B198" s="1">
-        <v>0</v>
-      </c>
-      <c r="C198" s="1">
-        <v>1</v>
-      </c>
-      <c r="D198" s="1">
-        <v>0</v>
-      </c>
-      <c r="E198" s="1">
-        <v>0</v>
-      </c>
-      <c r="F198" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="199" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A199" s="3" t="s">
-        <v>204</v>
-      </c>
-      <c r="B199" s="1">
-        <v>1</v>
-      </c>
-      <c r="C199" s="1">
-        <v>1</v>
-      </c>
-      <c r="D199" s="1">
-        <v>0</v>
-      </c>
-      <c r="E199" s="1">
-        <v>0</v>
-      </c>
-      <c r="F199" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="200" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A200" s="3" t="s">
-        <v>205</v>
-      </c>
-      <c r="B200" s="1">
-        <v>1</v>
-      </c>
-      <c r="C200" s="1">
-        <v>1</v>
-      </c>
-      <c r="D200" s="1">
-        <v>0</v>
-      </c>
-      <c r="E200" s="1">
-        <v>0</v>
-      </c>
-      <c r="F200" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="201" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A201" s="3" t="s">
-        <v>206</v>
-      </c>
-      <c r="B201" s="1">
-        <v>1</v>
-      </c>
-      <c r="C201" s="1">
-        <v>1</v>
-      </c>
-      <c r="D201" s="1">
-        <v>0</v>
-      </c>
-      <c r="E201" s="1">
-        <v>0</v>
-      </c>
-      <c r="F201" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="202" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A202" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="B202" s="1">
-        <v>1</v>
-      </c>
-      <c r="C202" s="1">
-        <v>1</v>
-      </c>
-      <c r="D202" s="1">
-        <v>0</v>
-      </c>
-      <c r="E202" s="1">
-        <v>0</v>
-      </c>
-      <c r="F202" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="203" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A203" s="3" t="s">
-        <v>207</v>
-      </c>
-      <c r="B203" s="1">
-        <v>1</v>
-      </c>
-      <c r="C203" s="1">
-        <v>1</v>
-      </c>
-      <c r="D203" s="1">
-        <v>0</v>
-      </c>
-      <c r="E203" s="1">
-        <v>0</v>
-      </c>
-      <c r="F203" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="204" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A204" s="3" t="s">
-        <v>208</v>
-      </c>
-      <c r="B204" s="1">
-        <v>1</v>
-      </c>
-      <c r="C204" s="1">
-        <v>1</v>
-      </c>
-      <c r="D204" s="1">
-        <v>0</v>
-      </c>
-      <c r="E204" s="1">
-        <v>0</v>
-      </c>
-      <c r="F204" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="205" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A205" s="3" t="s">
-        <v>209</v>
-      </c>
-      <c r="B205" s="1">
-        <v>1</v>
-      </c>
-      <c r="C205" s="1">
-        <v>1</v>
-      </c>
-      <c r="D205" s="1">
-        <v>0</v>
-      </c>
-      <c r="E205" s="1">
-        <v>0</v>
-      </c>
-      <c r="F205" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="206" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A206" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="B206" s="1">
-        <v>1</v>
-      </c>
-      <c r="C206" s="1">
-        <v>1</v>
-      </c>
-      <c r="D206" s="1">
-        <v>0</v>
-      </c>
-      <c r="E206" s="1">
-        <v>0</v>
-      </c>
-      <c r="F206" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="207" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A207" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="B207" s="1">
-        <v>0</v>
-      </c>
-      <c r="C207" s="1">
-        <v>1</v>
-      </c>
-      <c r="D207" s="1">
-        <v>0</v>
-      </c>
-      <c r="E207" s="1">
-        <v>0</v>
-      </c>
-      <c r="F207" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="208" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A208" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="B208" s="1">
-        <v>1</v>
-      </c>
-      <c r="C208" s="1">
-        <v>0</v>
-      </c>
-      <c r="D208" s="1">
-        <v>0</v>
-      </c>
-      <c r="E208" s="1">
-        <v>0</v>
-      </c>
-      <c r="F208" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="209" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A209" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="B209" s="1">
-        <v>1</v>
-      </c>
-      <c r="C209" s="1">
-        <v>1</v>
-      </c>
-      <c r="D209" s="1">
-        <v>0</v>
-      </c>
-      <c r="E209" s="1">
-        <v>0</v>
-      </c>
-      <c r="F209" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="210" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A210" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="B210" s="1">
-        <v>1</v>
-      </c>
-      <c r="C210" s="1">
-        <v>1</v>
-      </c>
-      <c r="D210" s="1">
-        <v>0</v>
-      </c>
-      <c r="E210" s="1">
-        <v>0</v>
-      </c>
-      <c r="F210" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>